<commit_message>
fix: keep the products list's "Load more" count in the URL so Back from a product page returns to the same list and scroll position
</commit_message>
<xml_diff>
--- a/outputs/storage-solution-comparison/Inkarp_Storage_Solution_Comparison.xlsx
+++ b/outputs/storage-solution-comparison/Inkarp_Storage_Solution_Comparison.xlsx
@@ -665,12 +665,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -738,84 +732,17 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="22">
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
     <dxf>
       <font>
         <strike val="0"/>
@@ -1001,17 +928,39 @@
       </border>
     </dxf>
     <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
       <border>
         <top style="thin">
           <color indexed="64"/>
         </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
       </border>
     </dxf>
     <dxf>
@@ -1031,13 +980,55 @@
       </border>
     </dxf>
     <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <color theme="1"/>
+      </font>
       <fill>
         <patternFill>
           <fgColor indexed="64"/>
           <bgColor theme="0"/>
         </patternFill>
       </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
     </dxf>
     <dxf>
       <fill>
@@ -1137,6 +1128,45 @@
       </border>
     </dxf>
     <dxf>
+      <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
       <font>
         <strike val="0"/>
         <outline val="0"/>
@@ -1168,36 +1198,6 @@
         </horizontal>
       </border>
     </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1212,30 +1212,30 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="StorageSimpleGuide" displayName="StorageSimpleGuide" ref="A5:E21" totalsRowShown="0" headerRowDxfId="18" dataDxfId="12" headerRowBorderDxfId="20" tableBorderDxfId="21" totalsRowBorderDxfId="19">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="StorageSimpleGuide" displayName="StorageSimpleGuide" ref="A5:E21" totalsRowShown="0" headerRowDxfId="21" dataDxfId="19" headerRowBorderDxfId="20" tableBorderDxfId="18" totalsRowBorderDxfId="17">
   <autoFilter ref="A5:E21"/>
   <tableColumns count="5">
-    <tableColumn id="1" name="Topic" dataDxfId="17"/>
-    <tableColumn id="2" name="Simple explanation" dataDxfId="16"/>
-    <tableColumn id="3" name="Recommended choice" dataDxfId="15"/>
-    <tableColumn id="4" name="Example" dataDxfId="14"/>
-    <tableColumn id="5" name="Column1" dataDxfId="13"/>
+    <tableColumn id="1" name="Topic" dataDxfId="16"/>
+    <tableColumn id="2" name="Simple explanation" dataDxfId="15"/>
+    <tableColumn id="3" name="Recommended choice" dataDxfId="14"/>
+    <tableColumn id="4" name="Example" dataDxfId="13"/>
+    <tableColumn id="5" name="Column1" dataDxfId="12"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StorageSelectionChecklist" displayName="StorageSelectionChecklist" ref="A5:G27" totalsRowShown="0" headerRowDxfId="2" dataDxfId="1" headerRowBorderDxfId="10" tableBorderDxfId="11" totalsRowBorderDxfId="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StorageSelectionChecklist" displayName="StorageSelectionChecklist" ref="A5:G27" totalsRowShown="0" headerRowDxfId="11" dataDxfId="9" headerRowBorderDxfId="10" tableBorderDxfId="8" totalsRowBorderDxfId="7">
   <autoFilter ref="A5:G27"/>
   <tableColumns count="7">
-    <tableColumn id="1" name="No." dataDxfId="0"/>
-    <tableColumn id="2" name="Requirement to check" dataDxfId="8"/>
-    <tableColumn id="3" name="Why it matters" dataDxfId="7"/>
-    <tableColumn id="4" name="Recommended tool" dataDxfId="6"/>
-    <tableColumn id="5" name="Required?" dataDxfId="5"/>
-    <tableColumn id="6" name="Checked?" dataDxfId="4"/>
-    <tableColumn id="7" name="Notes / decision" dataDxfId="3"/>
+    <tableColumn id="1" name="No." dataDxfId="6"/>
+    <tableColumn id="2" name="Requirement to check" dataDxfId="5"/>
+    <tableColumn id="3" name="Why it matters" dataDxfId="4"/>
+    <tableColumn id="4" name="Recommended tool" dataDxfId="3"/>
+    <tableColumn id="5" name="Required?" dataDxfId="2"/>
+    <tableColumn id="6" name="Checked?" dataDxfId="1"/>
+    <tableColumn id="7" name="Notes / decision" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1457,24 +1457,24 @@
       <c r="H1" s="1"/>
     </row>
     <row r="2" spans="1:8" ht="21" x14ac:dyDescent="0.4">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="28" t="s">
         <v>78</v>
       </c>
-      <c r="B2" s="7"/>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="29" t="s">
         <v>79</v>
       </c>
-      <c r="B3" s="8"/>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
+      <c r="B3" s="29"/>
+      <c r="C3" s="29"/>
+      <c r="D3" s="29"/>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
@@ -1491,314 +1491,314 @@
       <c r="H4" s="1"/>
     </row>
     <row r="5" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="9" t="s">
+      <c r="A5" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="C5" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="D5" s="11" t="s">
+      <c r="D5" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="E5" s="12" t="s">
+      <c r="E5" s="8" t="s">
         <v>148</v>
       </c>
       <c r="F5" s="3"/>
       <c r="G5" s="3"/>
       <c r="H5" s="3"/>
     </row>
-    <row r="6" spans="1:8" s="17" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A6" s="13" t="s">
+    <row r="6" spans="1:8" s="13" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A6" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="B6" s="14" t="s">
+      <c r="B6" s="10" t="s">
         <v>85</v>
       </c>
-      <c r="C6" s="14" t="s">
+      <c r="C6" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="D6" s="15" t="s">
+      <c r="D6" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="E6" s="16"/>
-      <c r="F6" s="16"/>
-      <c r="G6" s="16"/>
-      <c r="H6" s="16"/>
-    </row>
-    <row r="7" spans="1:8" s="17" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A7" s="13" t="s">
+      <c r="E6" s="12"/>
+      <c r="F6" s="12"/>
+      <c r="G6" s="12"/>
+      <c r="H6" s="12"/>
+    </row>
+    <row r="7" spans="1:8" s="13" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A7" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="B7" s="14" t="s">
+      <c r="B7" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="C7" s="14" t="s">
+      <c r="C7" s="10" t="s">
         <v>90</v>
       </c>
-      <c r="D7" s="15" t="s">
+      <c r="D7" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="E7" s="16" t="s">
+      <c r="E7" s="12" t="s">
         <v>147</v>
       </c>
-      <c r="F7" s="16"/>
-      <c r="G7" s="16"/>
-      <c r="H7" s="16"/>
-    </row>
-    <row r="8" spans="1:8" s="17" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A8" s="13" t="s">
+      <c r="F7" s="12"/>
+      <c r="G7" s="12"/>
+      <c r="H7" s="12"/>
+    </row>
+    <row r="8" spans="1:8" s="13" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A8" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="B8" s="14" t="s">
+      <c r="B8" s="10" t="s">
         <v>93</v>
       </c>
-      <c r="C8" s="14" t="s">
+      <c r="C8" s="10" t="s">
         <v>94</v>
       </c>
-      <c r="D8" s="15" t="s">
+      <c r="D8" s="11" t="s">
         <v>95</v>
       </c>
-      <c r="E8" s="16"/>
-      <c r="F8" s="16"/>
-      <c r="G8" s="16"/>
-      <c r="H8" s="16"/>
-    </row>
-    <row r="9" spans="1:8" s="17" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A9" s="13" t="s">
+      <c r="E8" s="12"/>
+      <c r="F8" s="12"/>
+      <c r="G8" s="12"/>
+      <c r="H8" s="12"/>
+    </row>
+    <row r="9" spans="1:8" s="13" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A9" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="B9" s="14" t="s">
+      <c r="B9" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="C9" s="14" t="s">
+      <c r="C9" s="10" t="s">
         <v>97</v>
       </c>
-      <c r="D9" s="15" t="s">
+      <c r="D9" s="11" t="s">
         <v>98</v>
       </c>
-      <c r="E9" s="16"/>
-      <c r="F9" s="16"/>
-      <c r="G9" s="16"/>
-      <c r="H9" s="16"/>
-    </row>
-    <row r="10" spans="1:8" s="17" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A10" s="13" t="s">
+      <c r="E9" s="12"/>
+      <c r="F9" s="12"/>
+      <c r="G9" s="12"/>
+      <c r="H9" s="12"/>
+    </row>
+    <row r="10" spans="1:8" s="13" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A10" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="B10" s="14" t="s">
+      <c r="B10" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="C10" s="14" t="s">
+      <c r="C10" s="10" t="s">
         <v>101</v>
       </c>
-      <c r="D10" s="15" t="s">
+      <c r="D10" s="11" t="s">
         <v>102</v>
       </c>
-      <c r="E10" s="16"/>
-      <c r="F10" s="16"/>
-      <c r="G10" s="16"/>
-      <c r="H10" s="16"/>
-    </row>
-    <row r="11" spans="1:8" s="17" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A11" s="13" t="s">
+      <c r="E10" s="12"/>
+      <c r="F10" s="12"/>
+      <c r="G10" s="12"/>
+      <c r="H10" s="12"/>
+    </row>
+    <row r="11" spans="1:8" s="13" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A11" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="B11" s="14" t="s">
+      <c r="B11" s="10" t="s">
         <v>104</v>
       </c>
-      <c r="C11" s="14" t="s">
+      <c r="C11" s="10" t="s">
         <v>105</v>
       </c>
-      <c r="D11" s="15" t="s">
+      <c r="D11" s="11" t="s">
         <v>106</v>
       </c>
-      <c r="E11" s="16"/>
-      <c r="F11" s="16"/>
-      <c r="G11" s="16"/>
-      <c r="H11" s="16"/>
-    </row>
-    <row r="12" spans="1:8" s="17" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A12" s="13" t="s">
+      <c r="E11" s="12"/>
+      <c r="F11" s="12"/>
+      <c r="G11" s="12"/>
+      <c r="H11" s="12"/>
+    </row>
+    <row r="12" spans="1:8" s="13" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A12" s="9" t="s">
         <v>107</v>
       </c>
-      <c r="B12" s="14" t="s">
+      <c r="B12" s="10" t="s">
         <v>108</v>
       </c>
-      <c r="C12" s="14" t="s">
+      <c r="C12" s="10" t="s">
         <v>109</v>
       </c>
-      <c r="D12" s="15" t="s">
+      <c r="D12" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="E12" s="16"/>
-      <c r="F12" s="16"/>
-      <c r="G12" s="16"/>
-      <c r="H12" s="16"/>
-    </row>
-    <row r="13" spans="1:8" s="17" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A13" s="13" t="s">
+      <c r="E12" s="12"/>
+      <c r="F12" s="12"/>
+      <c r="G12" s="12"/>
+      <c r="H12" s="12"/>
+    </row>
+    <row r="13" spans="1:8" s="13" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A13" s="9" t="s">
         <v>111</v>
       </c>
-      <c r="B13" s="14" t="s">
+      <c r="B13" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="C13" s="14" t="s">
+      <c r="C13" s="10" t="s">
         <v>113</v>
       </c>
-      <c r="D13" s="15" t="s">
+      <c r="D13" s="11" t="s">
         <v>114</v>
       </c>
-      <c r="E13" s="16"/>
-      <c r="F13" s="16"/>
-      <c r="G13" s="16"/>
-      <c r="H13" s="16"/>
-    </row>
-    <row r="14" spans="1:8" s="17" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A14" s="13" t="s">
+      <c r="E13" s="12"/>
+      <c r="F13" s="12"/>
+      <c r="G13" s="12"/>
+      <c r="H13" s="12"/>
+    </row>
+    <row r="14" spans="1:8" s="13" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A14" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="B14" s="14" t="s">
+      <c r="B14" s="10" t="s">
         <v>116</v>
       </c>
-      <c r="C14" s="14" t="s">
+      <c r="C14" s="10" t="s">
         <v>117</v>
       </c>
-      <c r="D14" s="15" t="s">
+      <c r="D14" s="11" t="s">
         <v>118</v>
       </c>
-      <c r="E14" s="16"/>
-      <c r="F14" s="16"/>
-      <c r="G14" s="16"/>
-      <c r="H14" s="16"/>
-    </row>
-    <row r="15" spans="1:8" s="17" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A15" s="13" t="s">
+      <c r="E14" s="12"/>
+      <c r="F14" s="12"/>
+      <c r="G14" s="12"/>
+      <c r="H14" s="12"/>
+    </row>
+    <row r="15" spans="1:8" s="13" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A15" s="9" t="s">
         <v>119</v>
       </c>
-      <c r="B15" s="14" t="s">
+      <c r="B15" s="10" t="s">
         <v>120</v>
       </c>
-      <c r="C15" s="14" t="s">
+      <c r="C15" s="10" t="s">
         <v>121</v>
       </c>
-      <c r="D15" s="15" t="s">
+      <c r="D15" s="11" t="s">
         <v>122</v>
       </c>
-      <c r="E15" s="16"/>
-      <c r="F15" s="16"/>
-      <c r="G15" s="16"/>
-      <c r="H15" s="16"/>
-    </row>
-    <row r="16" spans="1:8" s="17" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A16" s="13" t="s">
+      <c r="E15" s="12"/>
+      <c r="F15" s="12"/>
+      <c r="G15" s="12"/>
+      <c r="H15" s="12"/>
+    </row>
+    <row r="16" spans="1:8" s="13" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A16" s="9" t="s">
         <v>123</v>
       </c>
-      <c r="B16" s="14" t="s">
+      <c r="B16" s="10" t="s">
         <v>124</v>
       </c>
-      <c r="C16" s="14" t="s">
+      <c r="C16" s="10" t="s">
         <v>125</v>
       </c>
-      <c r="D16" s="15" t="s">
+      <c r="D16" s="11" t="s">
         <v>126</v>
       </c>
-      <c r="E16" s="16"/>
-      <c r="F16" s="16"/>
-      <c r="G16" s="16"/>
-      <c r="H16" s="16"/>
-    </row>
-    <row r="17" spans="1:8" s="17" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A17" s="13" t="s">
+      <c r="E16" s="12"/>
+      <c r="F16" s="12"/>
+      <c r="G16" s="12"/>
+      <c r="H16" s="12"/>
+    </row>
+    <row r="17" spans="1:8" s="13" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A17" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="B17" s="14" t="s">
+      <c r="B17" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="C17" s="14" t="s">
+      <c r="C17" s="10" t="s">
         <v>129</v>
       </c>
-      <c r="D17" s="15" t="s">
+      <c r="D17" s="11" t="s">
         <v>130</v>
       </c>
-      <c r="E17" s="16"/>
-      <c r="F17" s="16"/>
-      <c r="G17" s="16"/>
-      <c r="H17" s="16"/>
-    </row>
-    <row r="18" spans="1:8" s="17" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A18" s="13" t="s">
+      <c r="E17" s="12"/>
+      <c r="F17" s="12"/>
+      <c r="G17" s="12"/>
+      <c r="H17" s="12"/>
+    </row>
+    <row r="18" spans="1:8" s="13" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A18" s="9" t="s">
         <v>131</v>
       </c>
-      <c r="B18" s="14" t="s">
+      <c r="B18" s="10" t="s">
         <v>132</v>
       </c>
-      <c r="C18" s="14" t="s">
+      <c r="C18" s="10" t="s">
         <v>133</v>
       </c>
-      <c r="D18" s="15" t="s">
+      <c r="D18" s="11" t="s">
         <v>134</v>
       </c>
-      <c r="E18" s="16"/>
-      <c r="F18" s="16"/>
-      <c r="G18" s="16"/>
-      <c r="H18" s="16"/>
-    </row>
-    <row r="19" spans="1:8" s="17" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A19" s="13" t="s">
+      <c r="E18" s="12"/>
+      <c r="F18" s="12"/>
+      <c r="G18" s="12"/>
+      <c r="H18" s="12"/>
+    </row>
+    <row r="19" spans="1:8" s="13" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A19" s="9" t="s">
         <v>135</v>
       </c>
-      <c r="B19" s="14" t="s">
+      <c r="B19" s="10" t="s">
         <v>136</v>
       </c>
-      <c r="C19" s="14" t="s">
+      <c r="C19" s="10" t="s">
         <v>137</v>
       </c>
-      <c r="D19" s="15" t="s">
+      <c r="D19" s="11" t="s">
         <v>138</v>
       </c>
-      <c r="E19" s="16"/>
-      <c r="F19" s="16"/>
-      <c r="G19" s="16"/>
-      <c r="H19" s="16"/>
-    </row>
-    <row r="20" spans="1:8" s="17" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A20" s="13" t="s">
+      <c r="E19" s="12"/>
+      <c r="F19" s="12"/>
+      <c r="G19" s="12"/>
+      <c r="H19" s="12"/>
+    </row>
+    <row r="20" spans="1:8" s="13" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A20" s="9" t="s">
         <v>139</v>
       </c>
-      <c r="B20" s="14" t="s">
+      <c r="B20" s="10" t="s">
         <v>140</v>
       </c>
-      <c r="C20" s="14" t="s">
+      <c r="C20" s="10" t="s">
         <v>141</v>
       </c>
-      <c r="D20" s="15" t="s">
+      <c r="D20" s="11" t="s">
         <v>142</v>
       </c>
-      <c r="E20" s="16"/>
-      <c r="F20" s="16"/>
-      <c r="G20" s="16"/>
-      <c r="H20" s="16"/>
-    </row>
-    <row r="21" spans="1:8" s="17" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A21" s="18" t="s">
+      <c r="E20" s="12"/>
+      <c r="F20" s="12"/>
+      <c r="G20" s="12"/>
+      <c r="H20" s="12"/>
+    </row>
+    <row r="21" spans="1:8" s="13" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A21" s="14" t="s">
         <v>143</v>
       </c>
-      <c r="B21" s="19" t="s">
+      <c r="B21" s="15" t="s">
         <v>144</v>
       </c>
-      <c r="C21" s="19" t="s">
+      <c r="C21" s="15" t="s">
         <v>145</v>
       </c>
-      <c r="D21" s="20" t="s">
+      <c r="D21" s="16" t="s">
         <v>146</v>
       </c>
-      <c r="E21" s="16"/>
-      <c r="F21" s="16"/>
-      <c r="G21" s="16"/>
-      <c r="H21" s="16"/>
+      <c r="E21" s="12"/>
+      <c r="F21" s="12"/>
+      <c r="G21" s="12"/>
+      <c r="H21" s="12"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
@@ -3608,7 +3608,7 @@
   <dimension ref="A1:H200"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="6.21875" style="31" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.21875" style="27" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="42" style="4" customWidth="1"/>
     <col min="3" max="3" width="50" style="4" customWidth="1"/>
     <col min="4" max="4" width="45" style="4" customWidth="1"/>
@@ -3619,7 +3619,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="28"/>
+      <c r="A1" s="24"/>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
@@ -3629,31 +3629,31 @@
       <c r="H1" s="3"/>
     </row>
     <row r="2" spans="1:8" ht="21" x14ac:dyDescent="0.4">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="30" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
       <c r="H2" s="3"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="6"/>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
-      <c r="E3" s="6"/>
-      <c r="F3" s="6"/>
-      <c r="G3" s="6"/>
+      <c r="B3" s="31"/>
+      <c r="C3" s="31"/>
+      <c r="D3" s="31"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="31"/>
+      <c r="G3" s="31"/>
       <c r="H3" s="3"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="28"/>
+      <c r="A4" s="24"/>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
@@ -3663,515 +3663,515 @@
       <c r="H4" s="3"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="21" t="s">
+      <c r="A5" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="22" t="s">
+      <c r="B5" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="22" t="s">
+      <c r="C5" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="22" t="s">
+      <c r="D5" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="E5" s="22" t="s">
+      <c r="E5" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="F5" s="22" t="s">
+      <c r="F5" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="G5" s="23" t="s">
+      <c r="G5" s="19" t="s">
         <v>8</v>
       </c>
       <c r="H5" s="3"/>
     </row>
     <row r="6" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A6" s="29">
+      <c r="A6" s="25">
         <v>1</v>
       </c>
-      <c r="B6" s="24" t="s">
+      <c r="B6" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="24" t="s">
+      <c r="C6" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="24" t="s">
+      <c r="D6" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="E6" s="24" t="s">
+      <c r="E6" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="F6" s="24" t="s">
+      <c r="F6" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="G6" s="25"/>
+      <c r="G6" s="21"/>
       <c r="H6" s="3"/>
     </row>
     <row r="7" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A7" s="29">
+      <c r="A7" s="25">
         <v>2</v>
       </c>
-      <c r="B7" s="24" t="s">
+      <c r="B7" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="24" t="s">
+      <c r="C7" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="D7" s="24" t="s">
+      <c r="D7" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="E7" s="24" t="s">
+      <c r="E7" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="F7" s="24" t="s">
+      <c r="F7" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="G7" s="25"/>
+      <c r="G7" s="21"/>
       <c r="H7" s="3"/>
     </row>
     <row r="8" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A8" s="29">
+      <c r="A8" s="25">
         <v>3</v>
       </c>
-      <c r="B8" s="24" t="s">
+      <c r="B8" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="C8" s="24" t="s">
+      <c r="C8" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="D8" s="24" t="s">
+      <c r="D8" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="E8" s="24" t="s">
+      <c r="E8" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="F8" s="24" t="s">
+      <c r="F8" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="G8" s="25"/>
+      <c r="G8" s="21"/>
       <c r="H8" s="3"/>
     </row>
     <row r="9" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A9" s="29">
+      <c r="A9" s="25">
         <v>4</v>
       </c>
-      <c r="B9" s="24" t="s">
+      <c r="B9" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="C9" s="24" t="s">
+      <c r="C9" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="D9" s="24" t="s">
+      <c r="D9" s="20" t="s">
         <v>22</v>
       </c>
-      <c r="E9" s="24" t="s">
+      <c r="E9" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="F9" s="24" t="s">
+      <c r="F9" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="G9" s="25"/>
+      <c r="G9" s="21"/>
       <c r="H9" s="3"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10" s="29">
+      <c r="A10" s="25">
         <v>5</v>
       </c>
-      <c r="B10" s="24" t="s">
+      <c r="B10" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="C10" s="24" t="s">
+      <c r="C10" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="D10" s="24" t="s">
+      <c r="D10" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="E10" s="24" t="s">
+      <c r="E10" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="F10" s="24" t="s">
+      <c r="F10" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="G10" s="25"/>
+      <c r="G10" s="21"/>
       <c r="H10" s="3"/>
     </row>
     <row r="11" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A11" s="29">
+      <c r="A11" s="25">
         <v>6</v>
       </c>
-      <c r="B11" s="24" t="s">
+      <c r="B11" s="20" t="s">
         <v>26</v>
       </c>
-      <c r="C11" s="24" t="s">
+      <c r="C11" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="D11" s="24" t="s">
+      <c r="D11" s="20" t="s">
         <v>28</v>
       </c>
-      <c r="E11" s="24" t="s">
+      <c r="E11" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="F11" s="24" t="s">
+      <c r="F11" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="G11" s="25"/>
+      <c r="G11" s="21"/>
       <c r="H11" s="3"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A12" s="29">
+      <c r="A12" s="25">
         <v>7</v>
       </c>
-      <c r="B12" s="24" t="s">
+      <c r="B12" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="C12" s="24" t="s">
+      <c r="C12" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="D12" s="24" t="s">
+      <c r="D12" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="E12" s="24" t="s">
+      <c r="E12" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="F12" s="24" t="s">
+      <c r="F12" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="G12" s="25"/>
+      <c r="G12" s="21"/>
       <c r="H12" s="3"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A13" s="29">
+      <c r="A13" s="25">
         <v>8</v>
       </c>
-      <c r="B13" s="24" t="s">
+      <c r="B13" s="20" t="s">
         <v>32</v>
       </c>
-      <c r="C13" s="24" t="s">
+      <c r="C13" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="D13" s="24" t="s">
+      <c r="D13" s="20" t="s">
         <v>34</v>
       </c>
-      <c r="E13" s="24" t="s">
+      <c r="E13" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="F13" s="24" t="s">
+      <c r="F13" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="G13" s="25"/>
+      <c r="G13" s="21"/>
       <c r="H13" s="3"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A14" s="29">
+      <c r="A14" s="25">
         <v>9</v>
       </c>
-      <c r="B14" s="24" t="s">
+      <c r="B14" s="20" t="s">
         <v>35</v>
       </c>
-      <c r="C14" s="24" t="s">
+      <c r="C14" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="D14" s="24" t="s">
+      <c r="D14" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="E14" s="24" t="s">
+      <c r="E14" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="F14" s="24" t="s">
+      <c r="F14" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="G14" s="25"/>
+      <c r="G14" s="21"/>
       <c r="H14" s="3"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A15" s="29">
+      <c r="A15" s="25">
         <v>10</v>
       </c>
-      <c r="B15" s="24" t="s">
+      <c r="B15" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="C15" s="24" t="s">
+      <c r="C15" s="20" t="s">
         <v>39</v>
       </c>
-      <c r="D15" s="24" t="s">
+      <c r="D15" s="20" t="s">
         <v>40</v>
       </c>
-      <c r="E15" s="24" t="s">
+      <c r="E15" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="F15" s="24" t="s">
+      <c r="F15" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="G15" s="25"/>
+      <c r="G15" s="21"/>
       <c r="H15" s="3"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A16" s="29">
+      <c r="A16" s="25">
         <v>11</v>
       </c>
-      <c r="B16" s="24" t="s">
+      <c r="B16" s="20" t="s">
         <v>41</v>
       </c>
-      <c r="C16" s="24" t="s">
+      <c r="C16" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="D16" s="24" t="s">
+      <c r="D16" s="20" t="s">
         <v>43</v>
       </c>
-      <c r="E16" s="24" t="s">
+      <c r="E16" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="F16" s="24" t="s">
+      <c r="F16" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="G16" s="25"/>
+      <c r="G16" s="21"/>
       <c r="H16" s="3"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A17" s="29">
+      <c r="A17" s="25">
         <v>12</v>
       </c>
-      <c r="B17" s="24" t="s">
+      <c r="B17" s="20" t="s">
         <v>44</v>
       </c>
-      <c r="C17" s="24" t="s">
+      <c r="C17" s="20" t="s">
         <v>45</v>
       </c>
-      <c r="D17" s="24" t="s">
+      <c r="D17" s="20" t="s">
         <v>46</v>
       </c>
-      <c r="E17" s="24" t="s">
+      <c r="E17" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="F17" s="24" t="s">
+      <c r="F17" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="G17" s="25"/>
+      <c r="G17" s="21"/>
       <c r="H17" s="3"/>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A18" s="29">
+      <c r="A18" s="25">
         <v>13</v>
       </c>
-      <c r="B18" s="24" t="s">
+      <c r="B18" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="C18" s="24" t="s">
+      <c r="C18" s="20" t="s">
         <v>48</v>
       </c>
-      <c r="D18" s="24" t="s">
+      <c r="D18" s="20" t="s">
         <v>49</v>
       </c>
-      <c r="E18" s="24" t="s">
+      <c r="E18" s="20" t="s">
         <v>50</v>
       </c>
-      <c r="F18" s="24" t="s">
+      <c r="F18" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="G18" s="25"/>
+      <c r="G18" s="21"/>
       <c r="H18" s="3"/>
     </row>
     <row r="19" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A19" s="29">
+      <c r="A19" s="25">
         <v>14</v>
       </c>
-      <c r="B19" s="24" t="s">
+      <c r="B19" s="20" t="s">
         <v>51</v>
       </c>
-      <c r="C19" s="24" t="s">
+      <c r="C19" s="20" t="s">
         <v>52</v>
       </c>
-      <c r="D19" s="24" t="s">
+      <c r="D19" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="E19" s="24" t="s">
+      <c r="E19" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="F19" s="24" t="s">
+      <c r="F19" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="G19" s="25"/>
+      <c r="G19" s="21"/>
       <c r="H19" s="3"/>
     </row>
     <row r="20" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A20" s="29">
+      <c r="A20" s="25">
         <v>15</v>
       </c>
-      <c r="B20" s="24" t="s">
+      <c r="B20" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="C20" s="24" t="s">
+      <c r="C20" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="D20" s="24" t="s">
+      <c r="D20" s="20" t="s">
         <v>56</v>
       </c>
-      <c r="E20" s="24" t="s">
+      <c r="E20" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="F20" s="24" t="s">
+      <c r="F20" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="G20" s="25"/>
+      <c r="G20" s="21"/>
       <c r="H20" s="3"/>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A21" s="29">
+      <c r="A21" s="25">
         <v>16</v>
       </c>
-      <c r="B21" s="24" t="s">
+      <c r="B21" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="C21" s="24" t="s">
+      <c r="C21" s="20" t="s">
         <v>58</v>
       </c>
-      <c r="D21" s="24" t="s">
+      <c r="D21" s="20" t="s">
         <v>59</v>
       </c>
-      <c r="E21" s="24" t="s">
+      <c r="E21" s="20" t="s">
         <v>50</v>
       </c>
-      <c r="F21" s="24" t="s">
+      <c r="F21" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="G21" s="25"/>
+      <c r="G21" s="21"/>
       <c r="H21" s="3"/>
     </row>
     <row r="22" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A22" s="29">
+      <c r="A22" s="25">
         <v>17</v>
       </c>
-      <c r="B22" s="24" t="s">
+      <c r="B22" s="20" t="s">
         <v>60</v>
       </c>
-      <c r="C22" s="24" t="s">
+      <c r="C22" s="20" t="s">
         <v>61</v>
       </c>
-      <c r="D22" s="24" t="s">
+      <c r="D22" s="20" t="s">
         <v>62</v>
       </c>
-      <c r="E22" s="24" t="s">
+      <c r="E22" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="F22" s="24" t="s">
+      <c r="F22" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="G22" s="25"/>
+      <c r="G22" s="21"/>
       <c r="H22" s="3"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A23" s="29">
+      <c r="A23" s="25">
         <v>18</v>
       </c>
-      <c r="B23" s="24" t="s">
+      <c r="B23" s="20" t="s">
         <v>63</v>
       </c>
-      <c r="C23" s="24" t="s">
+      <c r="C23" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="D23" s="24" t="s">
+      <c r="D23" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="E23" s="24" t="s">
+      <c r="E23" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="F23" s="24" t="s">
+      <c r="F23" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="G23" s="25"/>
+      <c r="G23" s="21"/>
       <c r="H23" s="3"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A24" s="29">
+      <c r="A24" s="25">
         <v>19</v>
       </c>
-      <c r="B24" s="24" t="s">
+      <c r="B24" s="20" t="s">
         <v>66</v>
       </c>
-      <c r="C24" s="24" t="s">
+      <c r="C24" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="D24" s="24" t="s">
+      <c r="D24" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="E24" s="24" t="s">
+      <c r="E24" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="F24" s="24" t="s">
+      <c r="F24" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="G24" s="25"/>
+      <c r="G24" s="21"/>
       <c r="H24" s="3"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A25" s="29">
+      <c r="A25" s="25">
         <v>20</v>
       </c>
-      <c r="B25" s="24" t="s">
+      <c r="B25" s="20" t="s">
         <v>69</v>
       </c>
-      <c r="C25" s="24" t="s">
+      <c r="C25" s="20" t="s">
         <v>70</v>
       </c>
-      <c r="D25" s="24" t="s">
+      <c r="D25" s="20" t="s">
         <v>71</v>
       </c>
-      <c r="E25" s="24" t="s">
+      <c r="E25" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="F25" s="24" t="s">
+      <c r="F25" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="G25" s="25"/>
+      <c r="G25" s="21"/>
       <c r="H25" s="3"/>
     </row>
     <row r="26" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A26" s="29">
+      <c r="A26" s="25">
         <v>21</v>
       </c>
-      <c r="B26" s="24" t="s">
+      <c r="B26" s="20" t="s">
         <v>72</v>
       </c>
-      <c r="C26" s="24" t="s">
+      <c r="C26" s="20" t="s">
         <v>73</v>
       </c>
-      <c r="D26" s="24" t="s">
+      <c r="D26" s="20" t="s">
         <v>74</v>
       </c>
-      <c r="E26" s="24" t="s">
+      <c r="E26" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="F26" s="24" t="s">
+      <c r="F26" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="G26" s="25"/>
+      <c r="G26" s="21"/>
       <c r="H26" s="3"/>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A27" s="30">
+      <c r="A27" s="26">
         <v>22</v>
       </c>
-      <c r="B27" s="26" t="s">
+      <c r="B27" s="22" t="s">
         <v>75</v>
       </c>
-      <c r="C27" s="26" t="s">
+      <c r="C27" s="22" t="s">
         <v>76</v>
       </c>
-      <c r="D27" s="26" t="s">
+      <c r="D27" s="22" t="s">
         <v>77</v>
       </c>
-      <c r="E27" s="26" t="s">
+      <c r="E27" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="F27" s="26" t="s">
+      <c r="F27" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="G27" s="27"/>
+      <c r="G27" s="23"/>
       <c r="H27" s="3"/>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A28" s="28"/>
+      <c r="A28" s="24"/>
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
       <c r="D28" s="3"/>
@@ -4181,7 +4181,7 @@
       <c r="H28" s="3"/>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A29" s="28"/>
+      <c r="A29" s="24"/>
       <c r="B29" s="3"/>
       <c r="C29" s="3"/>
       <c r="D29" s="3"/>
@@ -4191,7 +4191,7 @@
       <c r="H29" s="3"/>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A30" s="28"/>
+      <c r="A30" s="24"/>
       <c r="B30" s="3"/>
       <c r="C30" s="3"/>
       <c r="D30" s="3"/>
@@ -4201,7 +4201,7 @@
       <c r="H30" s="3"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A31" s="28"/>
+      <c r="A31" s="24"/>
       <c r="B31" s="3"/>
       <c r="C31" s="3"/>
       <c r="D31" s="3"/>
@@ -4211,7 +4211,7 @@
       <c r="H31" s="3"/>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A32" s="28"/>
+      <c r="A32" s="24"/>
       <c r="B32" s="3"/>
       <c r="C32" s="3"/>
       <c r="D32" s="3"/>
@@ -4221,7 +4221,7 @@
       <c r="H32" s="3"/>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A33" s="28"/>
+      <c r="A33" s="24"/>
       <c r="B33" s="3"/>
       <c r="C33" s="3"/>
       <c r="D33" s="3"/>
@@ -4231,7 +4231,7 @@
       <c r="H33" s="3"/>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A34" s="28"/>
+      <c r="A34" s="24"/>
       <c r="B34" s="3"/>
       <c r="C34" s="3"/>
       <c r="D34" s="3"/>
@@ -4241,7 +4241,7 @@
       <c r="H34" s="3"/>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A35" s="28"/>
+      <c r="A35" s="24"/>
       <c r="B35" s="3"/>
       <c r="C35" s="3"/>
       <c r="D35" s="3"/>
@@ -4251,7 +4251,7 @@
       <c r="H35" s="3"/>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A36" s="28"/>
+      <c r="A36" s="24"/>
       <c r="B36" s="3"/>
       <c r="C36" s="3"/>
       <c r="D36" s="3"/>
@@ -4261,7 +4261,7 @@
       <c r="H36" s="3"/>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A37" s="28"/>
+      <c r="A37" s="24"/>
       <c r="B37" s="3"/>
       <c r="C37" s="3"/>
       <c r="D37" s="3"/>
@@ -4271,7 +4271,7 @@
       <c r="H37" s="3"/>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A38" s="28"/>
+      <c r="A38" s="24"/>
       <c r="B38" s="3"/>
       <c r="C38" s="3"/>
       <c r="D38" s="3"/>
@@ -4281,7 +4281,7 @@
       <c r="H38" s="3"/>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A39" s="28"/>
+      <c r="A39" s="24"/>
       <c r="B39" s="3"/>
       <c r="C39" s="3"/>
       <c r="D39" s="3"/>
@@ -4291,7 +4291,7 @@
       <c r="H39" s="3"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A40" s="28"/>
+      <c r="A40" s="24"/>
       <c r="B40" s="3"/>
       <c r="C40" s="3"/>
       <c r="D40" s="3"/>
@@ -4301,7 +4301,7 @@
       <c r="H40" s="3"/>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A41" s="28"/>
+      <c r="A41" s="24"/>
       <c r="B41" s="3"/>
       <c r="C41" s="3"/>
       <c r="D41" s="3"/>
@@ -4311,7 +4311,7 @@
       <c r="H41" s="3"/>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A42" s="28"/>
+      <c r="A42" s="24"/>
       <c r="B42" s="3"/>
       <c r="C42" s="3"/>
       <c r="D42" s="3"/>
@@ -4321,7 +4321,7 @@
       <c r="H42" s="3"/>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A43" s="28"/>
+      <c r="A43" s="24"/>
       <c r="B43" s="3"/>
       <c r="C43" s="3"/>
       <c r="D43" s="3"/>
@@ -4331,7 +4331,7 @@
       <c r="H43" s="3"/>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A44" s="28"/>
+      <c r="A44" s="24"/>
       <c r="B44" s="3"/>
       <c r="C44" s="3"/>
       <c r="D44" s="3"/>
@@ -4341,7 +4341,7 @@
       <c r="H44" s="3"/>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A45" s="28"/>
+      <c r="A45" s="24"/>
       <c r="B45" s="3"/>
       <c r="C45" s="3"/>
       <c r="D45" s="3"/>
@@ -4351,7 +4351,7 @@
       <c r="H45" s="3"/>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A46" s="28"/>
+      <c r="A46" s="24"/>
       <c r="B46" s="3"/>
       <c r="C46" s="3"/>
       <c r="D46" s="3"/>
@@ -4361,7 +4361,7 @@
       <c r="H46" s="3"/>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A47" s="28"/>
+      <c r="A47" s="24"/>
       <c r="B47" s="3"/>
       <c r="C47" s="3"/>
       <c r="D47" s="3"/>
@@ -4371,7 +4371,7 @@
       <c r="H47" s="3"/>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A48" s="28"/>
+      <c r="A48" s="24"/>
       <c r="B48" s="3"/>
       <c r="C48" s="3"/>
       <c r="D48" s="3"/>
@@ -4381,7 +4381,7 @@
       <c r="H48" s="3"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A49" s="28"/>
+      <c r="A49" s="24"/>
       <c r="B49" s="3"/>
       <c r="C49" s="3"/>
       <c r="D49" s="3"/>
@@ -4391,7 +4391,7 @@
       <c r="H49" s="3"/>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A50" s="28"/>
+      <c r="A50" s="24"/>
       <c r="B50" s="3"/>
       <c r="C50" s="3"/>
       <c r="D50" s="3"/>
@@ -4401,7 +4401,7 @@
       <c r="H50" s="3"/>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A51" s="28"/>
+      <c r="A51" s="24"/>
       <c r="B51" s="3"/>
       <c r="C51" s="3"/>
       <c r="D51" s="3"/>
@@ -4411,7 +4411,7 @@
       <c r="H51" s="3"/>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A52" s="28"/>
+      <c r="A52" s="24"/>
       <c r="B52" s="3"/>
       <c r="C52" s="3"/>
       <c r="D52" s="3"/>
@@ -4421,7 +4421,7 @@
       <c r="H52" s="3"/>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A53" s="28"/>
+      <c r="A53" s="24"/>
       <c r="B53" s="3"/>
       <c r="C53" s="3"/>
       <c r="D53" s="3"/>
@@ -4431,7 +4431,7 @@
       <c r="H53" s="3"/>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A54" s="28"/>
+      <c r="A54" s="24"/>
       <c r="B54" s="3"/>
       <c r="C54" s="3"/>
       <c r="D54" s="3"/>
@@ -4441,7 +4441,7 @@
       <c r="H54" s="3"/>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A55" s="28"/>
+      <c r="A55" s="24"/>
       <c r="B55" s="3"/>
       <c r="C55" s="3"/>
       <c r="D55" s="3"/>
@@ -4451,7 +4451,7 @@
       <c r="H55" s="3"/>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A56" s="28"/>
+      <c r="A56" s="24"/>
       <c r="B56" s="3"/>
       <c r="C56" s="3"/>
       <c r="D56" s="3"/>
@@ -4461,7 +4461,7 @@
       <c r="H56" s="3"/>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A57" s="28"/>
+      <c r="A57" s="24"/>
       <c r="B57" s="3"/>
       <c r="C57" s="3"/>
       <c r="D57" s="3"/>
@@ -4471,7 +4471,7 @@
       <c r="H57" s="3"/>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A58" s="28"/>
+      <c r="A58" s="24"/>
       <c r="B58" s="3"/>
       <c r="C58" s="3"/>
       <c r="D58" s="3"/>
@@ -4481,7 +4481,7 @@
       <c r="H58" s="3"/>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A59" s="28"/>
+      <c r="A59" s="24"/>
       <c r="B59" s="3"/>
       <c r="C59" s="3"/>
       <c r="D59" s="3"/>
@@ -4491,7 +4491,7 @@
       <c r="H59" s="3"/>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A60" s="28"/>
+      <c r="A60" s="24"/>
       <c r="B60" s="3"/>
       <c r="C60" s="3"/>
       <c r="D60" s="3"/>
@@ -4501,7 +4501,7 @@
       <c r="H60" s="3"/>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A61" s="28"/>
+      <c r="A61" s="24"/>
       <c r="B61" s="3"/>
       <c r="C61" s="3"/>
       <c r="D61" s="3"/>
@@ -4511,7 +4511,7 @@
       <c r="H61" s="3"/>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A62" s="28"/>
+      <c r="A62" s="24"/>
       <c r="B62" s="3"/>
       <c r="C62" s="3"/>
       <c r="D62" s="3"/>
@@ -4521,7 +4521,7 @@
       <c r="H62" s="3"/>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A63" s="28"/>
+      <c r="A63" s="24"/>
       <c r="B63" s="3"/>
       <c r="C63" s="3"/>
       <c r="D63" s="3"/>
@@ -4531,7 +4531,7 @@
       <c r="H63" s="3"/>
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A64" s="28"/>
+      <c r="A64" s="24"/>
       <c r="B64" s="3"/>
       <c r="C64" s="3"/>
       <c r="D64" s="3"/>
@@ -4541,7 +4541,7 @@
       <c r="H64" s="3"/>
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A65" s="28"/>
+      <c r="A65" s="24"/>
       <c r="B65" s="3"/>
       <c r="C65" s="3"/>
       <c r="D65" s="3"/>
@@ -4551,7 +4551,7 @@
       <c r="H65" s="3"/>
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A66" s="28"/>
+      <c r="A66" s="24"/>
       <c r="B66" s="3"/>
       <c r="C66" s="3"/>
       <c r="D66" s="3"/>
@@ -4561,7 +4561,7 @@
       <c r="H66" s="3"/>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A67" s="28"/>
+      <c r="A67" s="24"/>
       <c r="B67" s="3"/>
       <c r="C67" s="3"/>
       <c r="D67" s="3"/>
@@ -4571,7 +4571,7 @@
       <c r="H67" s="3"/>
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A68" s="28"/>
+      <c r="A68" s="24"/>
       <c r="B68" s="3"/>
       <c r="C68" s="3"/>
       <c r="D68" s="3"/>
@@ -4581,7 +4581,7 @@
       <c r="H68" s="3"/>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A69" s="28"/>
+      <c r="A69" s="24"/>
       <c r="B69" s="3"/>
       <c r="C69" s="3"/>
       <c r="D69" s="3"/>
@@ -4591,7 +4591,7 @@
       <c r="H69" s="3"/>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A70" s="28"/>
+      <c r="A70" s="24"/>
       <c r="B70" s="3"/>
       <c r="C70" s="3"/>
       <c r="D70" s="3"/>
@@ -4601,7 +4601,7 @@
       <c r="H70" s="3"/>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A71" s="28"/>
+      <c r="A71" s="24"/>
       <c r="B71" s="3"/>
       <c r="C71" s="3"/>
       <c r="D71" s="3"/>
@@ -4611,7 +4611,7 @@
       <c r="H71" s="3"/>
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A72" s="28"/>
+      <c r="A72" s="24"/>
       <c r="B72" s="3"/>
       <c r="C72" s="3"/>
       <c r="D72" s="3"/>
@@ -4621,7 +4621,7 @@
       <c r="H72" s="3"/>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A73" s="28"/>
+      <c r="A73" s="24"/>
       <c r="B73" s="3"/>
       <c r="C73" s="3"/>
       <c r="D73" s="3"/>
@@ -4631,7 +4631,7 @@
       <c r="H73" s="3"/>
     </row>
     <row r="74" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A74" s="28"/>
+      <c r="A74" s="24"/>
       <c r="B74" s="3"/>
       <c r="C74" s="3"/>
       <c r="D74" s="3"/>
@@ -4641,7 +4641,7 @@
       <c r="H74" s="3"/>
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A75" s="28"/>
+      <c r="A75" s="24"/>
       <c r="B75" s="3"/>
       <c r="C75" s="3"/>
       <c r="D75" s="3"/>
@@ -4651,7 +4651,7 @@
       <c r="H75" s="3"/>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A76" s="28"/>
+      <c r="A76" s="24"/>
       <c r="B76" s="3"/>
       <c r="C76" s="3"/>
       <c r="D76" s="3"/>
@@ -4661,7 +4661,7 @@
       <c r="H76" s="3"/>
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A77" s="28"/>
+      <c r="A77" s="24"/>
       <c r="B77" s="3"/>
       <c r="C77" s="3"/>
       <c r="D77" s="3"/>
@@ -4671,7 +4671,7 @@
       <c r="H77" s="3"/>
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A78" s="28"/>
+      <c r="A78" s="24"/>
       <c r="B78" s="3"/>
       <c r="C78" s="3"/>
       <c r="D78" s="3"/>
@@ -4681,7 +4681,7 @@
       <c r="H78" s="3"/>
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A79" s="28"/>
+      <c r="A79" s="24"/>
       <c r="B79" s="3"/>
       <c r="C79" s="3"/>
       <c r="D79" s="3"/>
@@ -4691,7 +4691,7 @@
       <c r="H79" s="3"/>
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A80" s="28"/>
+      <c r="A80" s="24"/>
       <c r="B80" s="3"/>
       <c r="C80" s="3"/>
       <c r="D80" s="3"/>
@@ -4701,7 +4701,7 @@
       <c r="H80" s="3"/>
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A81" s="28"/>
+      <c r="A81" s="24"/>
       <c r="B81" s="3"/>
       <c r="C81" s="3"/>
       <c r="D81" s="3"/>
@@ -4711,7 +4711,7 @@
       <c r="H81" s="3"/>
     </row>
     <row r="82" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A82" s="28"/>
+      <c r="A82" s="24"/>
       <c r="B82" s="3"/>
       <c r="C82" s="3"/>
       <c r="D82" s="3"/>
@@ -4721,7 +4721,7 @@
       <c r="H82" s="3"/>
     </row>
     <row r="83" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A83" s="28"/>
+      <c r="A83" s="24"/>
       <c r="B83" s="3"/>
       <c r="C83" s="3"/>
       <c r="D83" s="3"/>
@@ -4731,7 +4731,7 @@
       <c r="H83" s="3"/>
     </row>
     <row r="84" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A84" s="28"/>
+      <c r="A84" s="24"/>
       <c r="B84" s="3"/>
       <c r="C84" s="3"/>
       <c r="D84" s="3"/>
@@ -4741,7 +4741,7 @@
       <c r="H84" s="3"/>
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A85" s="28"/>
+      <c r="A85" s="24"/>
       <c r="B85" s="3"/>
       <c r="C85" s="3"/>
       <c r="D85" s="3"/>
@@ -4751,7 +4751,7 @@
       <c r="H85" s="3"/>
     </row>
     <row r="86" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A86" s="28"/>
+      <c r="A86" s="24"/>
       <c r="B86" s="3"/>
       <c r="C86" s="3"/>
       <c r="D86" s="3"/>
@@ -4761,7 +4761,7 @@
       <c r="H86" s="3"/>
     </row>
     <row r="87" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A87" s="28"/>
+      <c r="A87" s="24"/>
       <c r="B87" s="3"/>
       <c r="C87" s="3"/>
       <c r="D87" s="3"/>
@@ -4771,7 +4771,7 @@
       <c r="H87" s="3"/>
     </row>
     <row r="88" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A88" s="28"/>
+      <c r="A88" s="24"/>
       <c r="B88" s="3"/>
       <c r="C88" s="3"/>
       <c r="D88" s="3"/>
@@ -4781,7 +4781,7 @@
       <c r="H88" s="3"/>
     </row>
     <row r="89" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A89" s="28"/>
+      <c r="A89" s="24"/>
       <c r="B89" s="3"/>
       <c r="C89" s="3"/>
       <c r="D89" s="3"/>
@@ -4791,7 +4791,7 @@
       <c r="H89" s="3"/>
     </row>
     <row r="90" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A90" s="28"/>
+      <c r="A90" s="24"/>
       <c r="B90" s="3"/>
       <c r="C90" s="3"/>
       <c r="D90" s="3"/>
@@ -4801,7 +4801,7 @@
       <c r="H90" s="3"/>
     </row>
     <row r="91" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A91" s="28"/>
+      <c r="A91" s="24"/>
       <c r="B91" s="3"/>
       <c r="C91" s="3"/>
       <c r="D91" s="3"/>
@@ -4811,7 +4811,7 @@
       <c r="H91" s="3"/>
     </row>
     <row r="92" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A92" s="28"/>
+      <c r="A92" s="24"/>
       <c r="B92" s="3"/>
       <c r="C92" s="3"/>
       <c r="D92" s="3"/>
@@ -4821,7 +4821,7 @@
       <c r="H92" s="3"/>
     </row>
     <row r="93" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A93" s="28"/>
+      <c r="A93" s="24"/>
       <c r="B93" s="3"/>
       <c r="C93" s="3"/>
       <c r="D93" s="3"/>
@@ -4831,7 +4831,7 @@
       <c r="H93" s="3"/>
     </row>
     <row r="94" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A94" s="28"/>
+      <c r="A94" s="24"/>
       <c r="B94" s="3"/>
       <c r="C94" s="3"/>
       <c r="D94" s="3"/>
@@ -4841,7 +4841,7 @@
       <c r="H94" s="3"/>
     </row>
     <row r="95" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A95" s="28"/>
+      <c r="A95" s="24"/>
       <c r="B95" s="3"/>
       <c r="C95" s="3"/>
       <c r="D95" s="3"/>
@@ -4851,7 +4851,7 @@
       <c r="H95" s="3"/>
     </row>
     <row r="96" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A96" s="28"/>
+      <c r="A96" s="24"/>
       <c r="B96" s="3"/>
       <c r="C96" s="3"/>
       <c r="D96" s="3"/>
@@ -4861,7 +4861,7 @@
       <c r="H96" s="3"/>
     </row>
     <row r="97" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A97" s="28"/>
+      <c r="A97" s="24"/>
       <c r="B97" s="3"/>
       <c r="C97" s="3"/>
       <c r="D97" s="3"/>
@@ -4871,7 +4871,7 @@
       <c r="H97" s="3"/>
     </row>
     <row r="98" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A98" s="28"/>
+      <c r="A98" s="24"/>
       <c r="B98" s="3"/>
       <c r="C98" s="3"/>
       <c r="D98" s="3"/>
@@ -4881,7 +4881,7 @@
       <c r="H98" s="3"/>
     </row>
     <row r="99" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A99" s="28"/>
+      <c r="A99" s="24"/>
       <c r="B99" s="3"/>
       <c r="C99" s="3"/>
       <c r="D99" s="3"/>
@@ -4891,7 +4891,7 @@
       <c r="H99" s="3"/>
     </row>
     <row r="100" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A100" s="28"/>
+      <c r="A100" s="24"/>
       <c r="B100" s="3"/>
       <c r="C100" s="3"/>
       <c r="D100" s="3"/>
@@ -4901,7 +4901,7 @@
       <c r="H100" s="3"/>
     </row>
     <row r="101" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A101" s="28"/>
+      <c r="A101" s="24"/>
       <c r="B101" s="3"/>
       <c r="C101" s="3"/>
       <c r="D101" s="3"/>
@@ -4911,7 +4911,7 @@
       <c r="H101" s="3"/>
     </row>
     <row r="102" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A102" s="28"/>
+      <c r="A102" s="24"/>
       <c r="B102" s="3"/>
       <c r="C102" s="3"/>
       <c r="D102" s="3"/>
@@ -4921,7 +4921,7 @@
       <c r="H102" s="3"/>
     </row>
     <row r="103" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A103" s="28"/>
+      <c r="A103" s="24"/>
       <c r="B103" s="3"/>
       <c r="C103" s="3"/>
       <c r="D103" s="3"/>
@@ -4931,7 +4931,7 @@
       <c r="H103" s="3"/>
     </row>
     <row r="104" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A104" s="28"/>
+      <c r="A104" s="24"/>
       <c r="B104" s="3"/>
       <c r="C104" s="3"/>
       <c r="D104" s="3"/>
@@ -4941,7 +4941,7 @@
       <c r="H104" s="3"/>
     </row>
     <row r="105" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A105" s="28"/>
+      <c r="A105" s="24"/>
       <c r="B105" s="3"/>
       <c r="C105" s="3"/>
       <c r="D105" s="3"/>
@@ -4951,7 +4951,7 @@
       <c r="H105" s="3"/>
     </row>
     <row r="106" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A106" s="28"/>
+      <c r="A106" s="24"/>
       <c r="B106" s="3"/>
       <c r="C106" s="3"/>
       <c r="D106" s="3"/>
@@ -4961,7 +4961,7 @@
       <c r="H106" s="3"/>
     </row>
     <row r="107" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A107" s="28"/>
+      <c r="A107" s="24"/>
       <c r="B107" s="3"/>
       <c r="C107" s="3"/>
       <c r="D107" s="3"/>
@@ -4971,7 +4971,7 @@
       <c r="H107" s="3"/>
     </row>
     <row r="108" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A108" s="28"/>
+      <c r="A108" s="24"/>
       <c r="B108" s="3"/>
       <c r="C108" s="3"/>
       <c r="D108" s="3"/>
@@ -4981,7 +4981,7 @@
       <c r="H108" s="3"/>
     </row>
     <row r="109" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A109" s="28"/>
+      <c r="A109" s="24"/>
       <c r="B109" s="3"/>
       <c r="C109" s="3"/>
       <c r="D109" s="3"/>
@@ -4991,7 +4991,7 @@
       <c r="H109" s="3"/>
     </row>
     <row r="110" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A110" s="28"/>
+      <c r="A110" s="24"/>
       <c r="B110" s="3"/>
       <c r="C110" s="3"/>
       <c r="D110" s="3"/>
@@ -5001,7 +5001,7 @@
       <c r="H110" s="3"/>
     </row>
     <row r="111" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A111" s="28"/>
+      <c r="A111" s="24"/>
       <c r="B111" s="3"/>
       <c r="C111" s="3"/>
       <c r="D111" s="3"/>
@@ -5011,7 +5011,7 @@
       <c r="H111" s="3"/>
     </row>
     <row r="112" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A112" s="28"/>
+      <c r="A112" s="24"/>
       <c r="B112" s="3"/>
       <c r="C112" s="3"/>
       <c r="D112" s="3"/>
@@ -5021,7 +5021,7 @@
       <c r="H112" s="3"/>
     </row>
     <row r="113" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A113" s="28"/>
+      <c r="A113" s="24"/>
       <c r="B113" s="3"/>
       <c r="C113" s="3"/>
       <c r="D113" s="3"/>
@@ -5031,7 +5031,7 @@
       <c r="H113" s="3"/>
     </row>
     <row r="114" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A114" s="28"/>
+      <c r="A114" s="24"/>
       <c r="B114" s="3"/>
       <c r="C114" s="3"/>
       <c r="D114" s="3"/>
@@ -5041,7 +5041,7 @@
       <c r="H114" s="3"/>
     </row>
     <row r="115" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A115" s="28"/>
+      <c r="A115" s="24"/>
       <c r="B115" s="3"/>
       <c r="C115" s="3"/>
       <c r="D115" s="3"/>
@@ -5051,7 +5051,7 @@
       <c r="H115" s="3"/>
     </row>
     <row r="116" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A116" s="28"/>
+      <c r="A116" s="24"/>
       <c r="B116" s="3"/>
       <c r="C116" s="3"/>
       <c r="D116" s="3"/>
@@ -5061,7 +5061,7 @@
       <c r="H116" s="3"/>
     </row>
     <row r="117" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A117" s="28"/>
+      <c r="A117" s="24"/>
       <c r="B117" s="3"/>
       <c r="C117" s="3"/>
       <c r="D117" s="3"/>
@@ -5071,7 +5071,7 @@
       <c r="H117" s="3"/>
     </row>
     <row r="118" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A118" s="28"/>
+      <c r="A118" s="24"/>
       <c r="B118" s="3"/>
       <c r="C118" s="3"/>
       <c r="D118" s="3"/>
@@ -5081,7 +5081,7 @@
       <c r="H118" s="3"/>
     </row>
     <row r="119" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A119" s="28"/>
+      <c r="A119" s="24"/>
       <c r="B119" s="3"/>
       <c r="C119" s="3"/>
       <c r="D119" s="3"/>
@@ -5091,7 +5091,7 @@
       <c r="H119" s="3"/>
     </row>
     <row r="120" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A120" s="28"/>
+      <c r="A120" s="24"/>
       <c r="B120" s="3"/>
       <c r="C120" s="3"/>
       <c r="D120" s="3"/>
@@ -5101,7 +5101,7 @@
       <c r="H120" s="3"/>
     </row>
     <row r="121" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A121" s="28"/>
+      <c r="A121" s="24"/>
       <c r="B121" s="3"/>
       <c r="C121" s="3"/>
       <c r="D121" s="3"/>
@@ -5111,7 +5111,7 @@
       <c r="H121" s="3"/>
     </row>
     <row r="122" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A122" s="28"/>
+      <c r="A122" s="24"/>
       <c r="B122" s="3"/>
       <c r="C122" s="3"/>
       <c r="D122" s="3"/>
@@ -5121,7 +5121,7 @@
       <c r="H122" s="3"/>
     </row>
     <row r="123" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A123" s="28"/>
+      <c r="A123" s="24"/>
       <c r="B123" s="3"/>
       <c r="C123" s="3"/>
       <c r="D123" s="3"/>
@@ -5131,7 +5131,7 @@
       <c r="H123" s="3"/>
     </row>
     <row r="124" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A124" s="28"/>
+      <c r="A124" s="24"/>
       <c r="B124" s="3"/>
       <c r="C124" s="3"/>
       <c r="D124" s="3"/>
@@ -5141,7 +5141,7 @@
       <c r="H124" s="3"/>
     </row>
     <row r="125" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A125" s="28"/>
+      <c r="A125" s="24"/>
       <c r="B125" s="3"/>
       <c r="C125" s="3"/>
       <c r="D125" s="3"/>
@@ -5151,7 +5151,7 @@
       <c r="H125" s="3"/>
     </row>
     <row r="126" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A126" s="28"/>
+      <c r="A126" s="24"/>
       <c r="B126" s="3"/>
       <c r="C126" s="3"/>
       <c r="D126" s="3"/>
@@ -5161,7 +5161,7 @@
       <c r="H126" s="3"/>
     </row>
     <row r="127" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A127" s="28"/>
+      <c r="A127" s="24"/>
       <c r="B127" s="3"/>
       <c r="C127" s="3"/>
       <c r="D127" s="3"/>
@@ -5171,7 +5171,7 @@
       <c r="H127" s="3"/>
     </row>
     <row r="128" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A128" s="28"/>
+      <c r="A128" s="24"/>
       <c r="B128" s="3"/>
       <c r="C128" s="3"/>
       <c r="D128" s="3"/>
@@ -5181,7 +5181,7 @@
       <c r="H128" s="3"/>
     </row>
     <row r="129" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A129" s="28"/>
+      <c r="A129" s="24"/>
       <c r="B129" s="3"/>
       <c r="C129" s="3"/>
       <c r="D129" s="3"/>
@@ -5191,7 +5191,7 @@
       <c r="H129" s="3"/>
     </row>
     <row r="130" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A130" s="28"/>
+      <c r="A130" s="24"/>
       <c r="B130" s="3"/>
       <c r="C130" s="3"/>
       <c r="D130" s="3"/>
@@ -5201,7 +5201,7 @@
       <c r="H130" s="3"/>
     </row>
     <row r="131" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A131" s="28"/>
+      <c r="A131" s="24"/>
       <c r="B131" s="3"/>
       <c r="C131" s="3"/>
       <c r="D131" s="3"/>
@@ -5211,7 +5211,7 @@
       <c r="H131" s="3"/>
     </row>
     <row r="132" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A132" s="28"/>
+      <c r="A132" s="24"/>
       <c r="B132" s="3"/>
       <c r="C132" s="3"/>
       <c r="D132" s="3"/>
@@ -5221,7 +5221,7 @@
       <c r="H132" s="3"/>
     </row>
     <row r="133" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A133" s="28"/>
+      <c r="A133" s="24"/>
       <c r="B133" s="3"/>
       <c r="C133" s="3"/>
       <c r="D133" s="3"/>
@@ -5231,7 +5231,7 @@
       <c r="H133" s="3"/>
     </row>
     <row r="134" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A134" s="28"/>
+      <c r="A134" s="24"/>
       <c r="B134" s="3"/>
       <c r="C134" s="3"/>
       <c r="D134" s="3"/>
@@ -5241,7 +5241,7 @@
       <c r="H134" s="3"/>
     </row>
     <row r="135" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A135" s="28"/>
+      <c r="A135" s="24"/>
       <c r="B135" s="3"/>
       <c r="C135" s="3"/>
       <c r="D135" s="3"/>
@@ -5251,7 +5251,7 @@
       <c r="H135" s="3"/>
     </row>
     <row r="136" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A136" s="28"/>
+      <c r="A136" s="24"/>
       <c r="B136" s="3"/>
       <c r="C136" s="3"/>
       <c r="D136" s="3"/>
@@ -5261,7 +5261,7 @@
       <c r="H136" s="3"/>
     </row>
     <row r="137" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A137" s="28"/>
+      <c r="A137" s="24"/>
       <c r="B137" s="3"/>
       <c r="C137" s="3"/>
       <c r="D137" s="3"/>
@@ -5271,7 +5271,7 @@
       <c r="H137" s="3"/>
     </row>
     <row r="138" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A138" s="28"/>
+      <c r="A138" s="24"/>
       <c r="B138" s="3"/>
       <c r="C138" s="3"/>
       <c r="D138" s="3"/>
@@ -5281,7 +5281,7 @@
       <c r="H138" s="3"/>
     </row>
     <row r="139" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A139" s="28"/>
+      <c r="A139" s="24"/>
       <c r="B139" s="3"/>
       <c r="C139" s="3"/>
       <c r="D139" s="3"/>
@@ -5291,7 +5291,7 @@
       <c r="H139" s="3"/>
     </row>
     <row r="140" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A140" s="28"/>
+      <c r="A140" s="24"/>
       <c r="B140" s="3"/>
       <c r="C140" s="3"/>
       <c r="D140" s="3"/>
@@ -5301,7 +5301,7 @@
       <c r="H140" s="3"/>
     </row>
     <row r="141" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A141" s="28"/>
+      <c r="A141" s="24"/>
       <c r="B141" s="3"/>
       <c r="C141" s="3"/>
       <c r="D141" s="3"/>
@@ -5311,7 +5311,7 @@
       <c r="H141" s="3"/>
     </row>
     <row r="142" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A142" s="28"/>
+      <c r="A142" s="24"/>
       <c r="B142" s="3"/>
       <c r="C142" s="3"/>
       <c r="D142" s="3"/>
@@ -5321,7 +5321,7 @@
       <c r="H142" s="3"/>
     </row>
     <row r="143" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A143" s="28"/>
+      <c r="A143" s="24"/>
       <c r="B143" s="3"/>
       <c r="C143" s="3"/>
       <c r="D143" s="3"/>
@@ -5331,7 +5331,7 @@
       <c r="H143" s="3"/>
     </row>
     <row r="144" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A144" s="28"/>
+      <c r="A144" s="24"/>
       <c r="B144" s="3"/>
       <c r="C144" s="3"/>
       <c r="D144" s="3"/>
@@ -5341,7 +5341,7 @@
       <c r="H144" s="3"/>
     </row>
     <row r="145" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A145" s="28"/>
+      <c r="A145" s="24"/>
       <c r="B145" s="3"/>
       <c r="C145" s="3"/>
       <c r="D145" s="3"/>
@@ -5351,7 +5351,7 @@
       <c r="H145" s="3"/>
     </row>
     <row r="146" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A146" s="28"/>
+      <c r="A146" s="24"/>
       <c r="B146" s="3"/>
       <c r="C146" s="3"/>
       <c r="D146" s="3"/>
@@ -5361,7 +5361,7 @@
       <c r="H146" s="3"/>
     </row>
     <row r="147" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A147" s="28"/>
+      <c r="A147" s="24"/>
       <c r="B147" s="3"/>
       <c r="C147" s="3"/>
       <c r="D147" s="3"/>
@@ -5371,7 +5371,7 @@
       <c r="H147" s="3"/>
     </row>
     <row r="148" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A148" s="28"/>
+      <c r="A148" s="24"/>
       <c r="B148" s="3"/>
       <c r="C148" s="3"/>
       <c r="D148" s="3"/>
@@ -5381,7 +5381,7 @@
       <c r="H148" s="3"/>
     </row>
     <row r="149" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A149" s="28"/>
+      <c r="A149" s="24"/>
       <c r="B149" s="3"/>
       <c r="C149" s="3"/>
       <c r="D149" s="3"/>
@@ -5391,7 +5391,7 @@
       <c r="H149" s="3"/>
     </row>
     <row r="150" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A150" s="28"/>
+      <c r="A150" s="24"/>
       <c r="B150" s="3"/>
       <c r="C150" s="3"/>
       <c r="D150" s="3"/>
@@ -5401,7 +5401,7 @@
       <c r="H150" s="3"/>
     </row>
     <row r="151" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A151" s="28"/>
+      <c r="A151" s="24"/>
       <c r="B151" s="3"/>
       <c r="C151" s="3"/>
       <c r="D151" s="3"/>
@@ -5411,7 +5411,7 @@
       <c r="H151" s="3"/>
     </row>
     <row r="152" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A152" s="28"/>
+      <c r="A152" s="24"/>
       <c r="B152" s="3"/>
       <c r="C152" s="3"/>
       <c r="D152" s="3"/>
@@ -5421,7 +5421,7 @@
       <c r="H152" s="3"/>
     </row>
     <row r="153" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A153" s="28"/>
+      <c r="A153" s="24"/>
       <c r="B153" s="3"/>
       <c r="C153" s="3"/>
       <c r="D153" s="3"/>
@@ -5431,7 +5431,7 @@
       <c r="H153" s="3"/>
     </row>
     <row r="154" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A154" s="28"/>
+      <c r="A154" s="24"/>
       <c r="B154" s="3"/>
       <c r="C154" s="3"/>
       <c r="D154" s="3"/>
@@ -5441,7 +5441,7 @@
       <c r="H154" s="3"/>
     </row>
     <row r="155" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A155" s="28"/>
+      <c r="A155" s="24"/>
       <c r="B155" s="3"/>
       <c r="C155" s="3"/>
       <c r="D155" s="3"/>
@@ -5451,7 +5451,7 @@
       <c r="H155" s="3"/>
     </row>
     <row r="156" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A156" s="28"/>
+      <c r="A156" s="24"/>
       <c r="B156" s="3"/>
       <c r="C156" s="3"/>
       <c r="D156" s="3"/>
@@ -5461,7 +5461,7 @@
       <c r="H156" s="3"/>
     </row>
     <row r="157" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A157" s="28"/>
+      <c r="A157" s="24"/>
       <c r="B157" s="3"/>
       <c r="C157" s="3"/>
       <c r="D157" s="3"/>
@@ -5471,7 +5471,7 @@
       <c r="H157" s="3"/>
     </row>
     <row r="158" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A158" s="28"/>
+      <c r="A158" s="24"/>
       <c r="B158" s="3"/>
       <c r="C158" s="3"/>
       <c r="D158" s="3"/>
@@ -5481,7 +5481,7 @@
       <c r="H158" s="3"/>
     </row>
     <row r="159" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A159" s="28"/>
+      <c r="A159" s="24"/>
       <c r="B159" s="3"/>
       <c r="C159" s="3"/>
       <c r="D159" s="3"/>
@@ -5491,7 +5491,7 @@
       <c r="H159" s="3"/>
     </row>
     <row r="160" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A160" s="28"/>
+      <c r="A160" s="24"/>
       <c r="B160" s="3"/>
       <c r="C160" s="3"/>
       <c r="D160" s="3"/>
@@ -5501,7 +5501,7 @@
       <c r="H160" s="3"/>
     </row>
     <row r="161" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A161" s="28"/>
+      <c r="A161" s="24"/>
       <c r="B161" s="3"/>
       <c r="C161" s="3"/>
       <c r="D161" s="3"/>
@@ -5511,7 +5511,7 @@
       <c r="H161" s="3"/>
     </row>
     <row r="162" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A162" s="28"/>
+      <c r="A162" s="24"/>
       <c r="B162" s="3"/>
       <c r="C162" s="3"/>
       <c r="D162" s="3"/>
@@ -5521,7 +5521,7 @@
       <c r="H162" s="3"/>
     </row>
     <row r="163" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A163" s="28"/>
+      <c r="A163" s="24"/>
       <c r="B163" s="3"/>
       <c r="C163" s="3"/>
       <c r="D163" s="3"/>
@@ -5531,7 +5531,7 @@
       <c r="H163" s="3"/>
     </row>
     <row r="164" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A164" s="28"/>
+      <c r="A164" s="24"/>
       <c r="B164" s="3"/>
       <c r="C164" s="3"/>
       <c r="D164" s="3"/>
@@ -5541,7 +5541,7 @@
       <c r="H164" s="3"/>
     </row>
     <row r="165" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A165" s="28"/>
+      <c r="A165" s="24"/>
       <c r="B165" s="3"/>
       <c r="C165" s="3"/>
       <c r="D165" s="3"/>
@@ -5551,7 +5551,7 @@
       <c r="H165" s="3"/>
     </row>
     <row r="166" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A166" s="28"/>
+      <c r="A166" s="24"/>
       <c r="B166" s="3"/>
       <c r="C166" s="3"/>
       <c r="D166" s="3"/>
@@ -5561,7 +5561,7 @@
       <c r="H166" s="3"/>
     </row>
     <row r="167" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A167" s="28"/>
+      <c r="A167" s="24"/>
       <c r="B167" s="3"/>
       <c r="C167" s="3"/>
       <c r="D167" s="3"/>
@@ -5571,7 +5571,7 @@
       <c r="H167" s="3"/>
     </row>
     <row r="168" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A168" s="28"/>
+      <c r="A168" s="24"/>
       <c r="B168" s="3"/>
       <c r="C168" s="3"/>
       <c r="D168" s="3"/>
@@ -5581,7 +5581,7 @@
       <c r="H168" s="3"/>
     </row>
     <row r="169" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A169" s="28"/>
+      <c r="A169" s="24"/>
       <c r="B169" s="3"/>
       <c r="C169" s="3"/>
       <c r="D169" s="3"/>
@@ -5591,7 +5591,7 @@
       <c r="H169" s="3"/>
     </row>
     <row r="170" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A170" s="28"/>
+      <c r="A170" s="24"/>
       <c r="B170" s="3"/>
       <c r="C170" s="3"/>
       <c r="D170" s="3"/>
@@ -5601,7 +5601,7 @@
       <c r="H170" s="3"/>
     </row>
     <row r="171" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A171" s="28"/>
+      <c r="A171" s="24"/>
       <c r="B171" s="3"/>
       <c r="C171" s="3"/>
       <c r="D171" s="3"/>
@@ -5611,7 +5611,7 @@
       <c r="H171" s="3"/>
     </row>
     <row r="172" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A172" s="28"/>
+      <c r="A172" s="24"/>
       <c r="B172" s="3"/>
       <c r="C172" s="3"/>
       <c r="D172" s="3"/>
@@ -5621,7 +5621,7 @@
       <c r="H172" s="3"/>
     </row>
     <row r="173" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A173" s="28"/>
+      <c r="A173" s="24"/>
       <c r="B173" s="3"/>
       <c r="C173" s="3"/>
       <c r="D173" s="3"/>
@@ -5631,7 +5631,7 @@
       <c r="H173" s="3"/>
     </row>
     <row r="174" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A174" s="28"/>
+      <c r="A174" s="24"/>
       <c r="B174" s="3"/>
       <c r="C174" s="3"/>
       <c r="D174" s="3"/>
@@ -5641,7 +5641,7 @@
       <c r="H174" s="3"/>
     </row>
     <row r="175" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A175" s="28"/>
+      <c r="A175" s="24"/>
       <c r="B175" s="3"/>
       <c r="C175" s="3"/>
       <c r="D175" s="3"/>
@@ -5651,7 +5651,7 @@
       <c r="H175" s="3"/>
     </row>
     <row r="176" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A176" s="28"/>
+      <c r="A176" s="24"/>
       <c r="B176" s="3"/>
       <c r="C176" s="3"/>
       <c r="D176" s="3"/>
@@ -5661,7 +5661,7 @@
       <c r="H176" s="3"/>
     </row>
     <row r="177" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A177" s="28"/>
+      <c r="A177" s="24"/>
       <c r="B177" s="3"/>
       <c r="C177" s="3"/>
       <c r="D177" s="3"/>
@@ -5671,7 +5671,7 @@
       <c r="H177" s="3"/>
     </row>
     <row r="178" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A178" s="28"/>
+      <c r="A178" s="24"/>
       <c r="B178" s="3"/>
       <c r="C178" s="3"/>
       <c r="D178" s="3"/>
@@ -5681,7 +5681,7 @@
       <c r="H178" s="3"/>
     </row>
     <row r="179" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A179" s="28"/>
+      <c r="A179" s="24"/>
       <c r="B179" s="3"/>
       <c r="C179" s="3"/>
       <c r="D179" s="3"/>
@@ -5691,7 +5691,7 @@
       <c r="H179" s="3"/>
     </row>
     <row r="180" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A180" s="28"/>
+      <c r="A180" s="24"/>
       <c r="B180" s="3"/>
       <c r="C180" s="3"/>
       <c r="D180" s="3"/>
@@ -5701,7 +5701,7 @@
       <c r="H180" s="3"/>
     </row>
     <row r="181" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A181" s="28"/>
+      <c r="A181" s="24"/>
       <c r="B181" s="3"/>
       <c r="C181" s="3"/>
       <c r="D181" s="3"/>
@@ -5711,7 +5711,7 @@
       <c r="H181" s="3"/>
     </row>
     <row r="182" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A182" s="28"/>
+      <c r="A182" s="24"/>
       <c r="B182" s="3"/>
       <c r="C182" s="3"/>
       <c r="D182" s="3"/>
@@ -5721,7 +5721,7 @@
       <c r="H182" s="3"/>
     </row>
     <row r="183" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A183" s="28"/>
+      <c r="A183" s="24"/>
       <c r="B183" s="3"/>
       <c r="C183" s="3"/>
       <c r="D183" s="3"/>
@@ -5731,7 +5731,7 @@
       <c r="H183" s="3"/>
     </row>
     <row r="184" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A184" s="28"/>
+      <c r="A184" s="24"/>
       <c r="B184" s="3"/>
       <c r="C184" s="3"/>
       <c r="D184" s="3"/>
@@ -5741,7 +5741,7 @@
       <c r="H184" s="3"/>
     </row>
     <row r="185" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A185" s="28"/>
+      <c r="A185" s="24"/>
       <c r="B185" s="3"/>
       <c r="C185" s="3"/>
       <c r="D185" s="3"/>
@@ -5751,7 +5751,7 @@
       <c r="H185" s="3"/>
     </row>
     <row r="186" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A186" s="28"/>
+      <c r="A186" s="24"/>
       <c r="B186" s="3"/>
       <c r="C186" s="3"/>
       <c r="D186" s="3"/>
@@ -5761,7 +5761,7 @@
       <c r="H186" s="3"/>
     </row>
     <row r="187" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A187" s="28"/>
+      <c r="A187" s="24"/>
       <c r="B187" s="3"/>
       <c r="C187" s="3"/>
       <c r="D187" s="3"/>
@@ -5771,7 +5771,7 @@
       <c r="H187" s="3"/>
     </row>
     <row r="188" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A188" s="28"/>
+      <c r="A188" s="24"/>
       <c r="B188" s="3"/>
       <c r="C188" s="3"/>
       <c r="D188" s="3"/>
@@ -5781,7 +5781,7 @@
       <c r="H188" s="3"/>
     </row>
     <row r="189" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A189" s="28"/>
+      <c r="A189" s="24"/>
       <c r="B189" s="3"/>
       <c r="C189" s="3"/>
       <c r="D189" s="3"/>
@@ -5791,7 +5791,7 @@
       <c r="H189" s="3"/>
     </row>
     <row r="190" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A190" s="28"/>
+      <c r="A190" s="24"/>
       <c r="B190" s="3"/>
       <c r="C190" s="3"/>
       <c r="D190" s="3"/>
@@ -5801,7 +5801,7 @@
       <c r="H190" s="3"/>
     </row>
     <row r="191" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A191" s="28"/>
+      <c r="A191" s="24"/>
       <c r="B191" s="3"/>
       <c r="C191" s="3"/>
       <c r="D191" s="3"/>
@@ -5811,7 +5811,7 @@
       <c r="H191" s="3"/>
     </row>
     <row r="192" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A192" s="28"/>
+      <c r="A192" s="24"/>
       <c r="B192" s="3"/>
       <c r="C192" s="3"/>
       <c r="D192" s="3"/>
@@ -5821,7 +5821,7 @@
       <c r="H192" s="3"/>
     </row>
     <row r="193" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A193" s="28"/>
+      <c r="A193" s="24"/>
       <c r="B193" s="3"/>
       <c r="C193" s="3"/>
       <c r="D193" s="3"/>
@@ -5831,7 +5831,7 @@
       <c r="H193" s="3"/>
     </row>
     <row r="194" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A194" s="28"/>
+      <c r="A194" s="24"/>
       <c r="B194" s="3"/>
       <c r="C194" s="3"/>
       <c r="D194" s="3"/>
@@ -5841,7 +5841,7 @@
       <c r="H194" s="3"/>
     </row>
     <row r="195" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A195" s="28"/>
+      <c r="A195" s="24"/>
       <c r="B195" s="3"/>
       <c r="C195" s="3"/>
       <c r="D195" s="3"/>
@@ -5851,7 +5851,7 @@
       <c r="H195" s="3"/>
     </row>
     <row r="196" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A196" s="28"/>
+      <c r="A196" s="24"/>
       <c r="B196" s="3"/>
       <c r="C196" s="3"/>
       <c r="D196" s="3"/>
@@ -5861,7 +5861,7 @@
       <c r="H196" s="3"/>
     </row>
     <row r="197" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A197" s="28"/>
+      <c r="A197" s="24"/>
       <c r="B197" s="3"/>
       <c r="C197" s="3"/>
       <c r="D197" s="3"/>
@@ -5871,7 +5871,7 @@
       <c r="H197" s="3"/>
     </row>
     <row r="198" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A198" s="28"/>
+      <c r="A198" s="24"/>
       <c r="B198" s="3"/>
       <c r="C198" s="3"/>
       <c r="D198" s="3"/>
@@ -5881,7 +5881,7 @@
       <c r="H198" s="3"/>
     </row>
     <row r="199" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A199" s="28"/>
+      <c r="A199" s="24"/>
       <c r="B199" s="3"/>
       <c r="C199" s="3"/>
       <c r="D199" s="3"/>
@@ -5891,7 +5891,7 @@
       <c r="H199" s="3"/>
     </row>
     <row r="200" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A200" s="28"/>
+      <c r="A200" s="24"/>
       <c r="B200" s="3"/>
       <c r="C200" s="3"/>
       <c r="D200" s="3"/>

</xml_diff>